<commit_message>
Publish Brandenburg_2016_MAR, Duisburg_2016_WC, Minsk_2016_JWCH, Moscow_2016_ECH
</commit_message>
<xml_diff>
--- a/events/Brandenburg_2016_MAR/Brandenburg_2016_MAR_Results.xlsx
+++ b/events/Brandenburg_2016_MAR/Brandenburg_2016_MAR_Results.xlsx
@@ -964,6 +964,11 @@
           <t>+03:47.060</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>65695</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3609,6 +3614,11 @@
           <t>+05:13.450</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>76936</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9452,6 +9462,11 @@
           <t>+01:40.380</t>
         </is>
       </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>94098</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -13168,6 +13183,11 @@
           <t>+01:20.730</t>
         </is>
       </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -18684,6 +18704,11 @@
       <c r="R258" t="inlineStr">
         <is>
           <t>66628</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>94098</t>
         </is>
       </c>
     </row>
@@ -25411,7 +25436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D361"/>
+  <dimension ref="A1:D365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33356,6 +33381,94 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>65695</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Anne Hauge</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>SØRENSEN</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>76936</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Anastasiia</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>YMELIANOVA</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>94098</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Jean</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>VAN DER WESTHUIZEN</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Kristina</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>BEDEC</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>